<commit_message>
Add Databricks E2E flow and column map to inventory UAT workbook
Cover Torsten's end-to-end request: real DBX objects/columns from MATDOC
through bridge_eu into France cube fields, plus richer backend logic on KPIs.

Co-authored-by: Akshay97 <axayteja_de@hotmail.com>
</commit_message>
<xml_diff>
--- a/Inventory_Testing.xlsx
+++ b/Inventory_Testing.xlsx
@@ -7,12 +7,14 @@
   </bookViews>
   <sheets>
     <sheet name="How to read (Torsten UAT)" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="KPIs List" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Issues Found" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="E2E Flow (DBX -&gt; Cube)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Column Map (DBX -&gt; Cube)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="KPIs List" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Issues Found" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'KPIs List'!$A$1:$F$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Issues Found'!$A$1:$K$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'KPIs List'!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Issues Found'!$A$1:$K$1</definedName>
   </definedNames>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
 </workbook>
@@ -105,7 +107,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -120,6 +122,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6EAF8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -165,7 +177,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -242,6 +254,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -622,7 +640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" style="16" min="1" max="1"/>
@@ -755,6 +773,42 @@
       <c r="B11" s="27" t="inlineStr">
         <is>
           <t>UDPEBP-323 Total Free Inventory mismatch; UDPEBP-324 assortment split; UDPEBP-325/328 Gross; special-stock discussion from 03-Aug daily call.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="55" customHeight="1" s="16">
+      <c r="A12" s="26" t="inlineStr">
+        <is>
+          <t>E2E Flow sheet</t>
+        </is>
+      </c>
+      <c r="B12" s="27" t="inlineStr">
+        <is>
+          <t>Step-by-step Databricks objects from SAP/MATDOC → silver → gold snapshot → bridge_eu → France cube partition → DAX measures. This is the flow Torsten asked for.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="55" customHeight="1" s="16">
+      <c r="A13" s="26" t="inlineStr">
+        <is>
+          <t>Column Map sheet</t>
+        </is>
+      </c>
+      <c r="B13" s="27" t="inlineStr">
+        <is>
+          <t>Exact cube field ↔ Databricks column mapping, including Inventory Type/Status/Special Stock formulas and which KPI uses them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="55" customHeight="1" s="16">
+      <c r="A14" s="26" t="inlineStr">
+        <is>
+          <t>Backend Logic column</t>
+        </is>
+      </c>
+      <c r="B14" s="27" t="inlineStr">
+        <is>
+          <t>Now includes real Databricks object/column names (not only business wording), plus plain English for UAT users.</t>
         </is>
       </c>
     </row>
@@ -767,6 +821,735 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" style="16" min="1" max="1"/>
+    <col width="45" customWidth="1" style="16" min="2" max="2"/>
+    <col width="50" customWidth="1" style="16" min="3" max="3"/>
+    <col width="55" customWidth="1" style="16" min="4" max="4"/>
+    <col width="40" customWidth="1" style="16" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="35" customHeight="1" s="16">
+      <c r="A1" s="28" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B1" s="28" t="inlineStr">
+        <is>
+          <t>Layer / Object (Databricks real names)</t>
+        </is>
+      </c>
+      <c r="C1" s="28" t="inlineStr">
+        <is>
+          <t>What happens (logic)</t>
+        </is>
+      </c>
+      <c r="D1" s="28" t="inlineStr">
+        <is>
+          <t>Key columns produced / used</t>
+        </is>
+      </c>
+      <c r="E1" s="28" t="inlineStr">
+        <is>
+          <t>Feeds cube field / filter</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="85" customHeight="1" s="16">
+      <c r="A2" s="36" t="inlineStr">
+        <is>
+          <t>1. SAP source</t>
+        </is>
+      </c>
+      <c r="B2" s="30" t="inlineStr">
+        <is>
+          <t>SAP S/4 MATDOC (+ ARUN allocation, STO, ATP sources)</t>
+        </is>
+      </c>
+      <c r="C2" s="30" t="inlineStr">
+        <is>
+          <t>Raw stock movements and related availability/allocation postings.</t>
+        </is>
+      </c>
+      <c r="D2" s="30" t="inlineStr">
+        <is>
+          <t>LBBSA_SID (stock type), SOBKZ (special stock), WERKS, LGORT, MATBF, MENGE/stock qty change, SGT_SCAT</t>
+        </is>
+      </c>
+      <c r="E2" s="30" t="inlineStr">
+        <is>
+          <t>Not in cube directly; compared manually in UAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="85" customHeight="1" s="16">
+      <c r="A3" s="36" t="inlineStr">
+        <is>
+          <t>2. Silver movements</t>
+        </is>
+      </c>
+      <c r="B3" s="30" t="inlineStr">
+        <is>
+          <t>s2_silver.fact_material_movements</t>
+        </is>
+      </c>
+      <c r="C3" s="30" t="inlineStr">
+        <is>
+          <t>Normalized MATDOC movements into Databricks.</t>
+        </is>
+      </c>
+      <c r="D3" s="30" t="inlineStr">
+        <is>
+          <t>company_code, plant, material, storage_location, stock_segment, stock_identifying_batch, inventory_special_stock_type, inventory_stock_type, matl_stk_change_qty_in_base_unit, posting_date</t>
+        </is>
+      </c>
+      <c r="E3" s="30" t="inlineStr">
+        <is>
+          <t>Basis for physical Inventory Type quantities</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="85" customHeight="1" s="16">
+      <c r="A4" s="36" t="inlineStr">
+        <is>
+          <t>3. Aggregate to stock-on-hand</t>
+        </is>
+      </c>
+      <c r="B4" s="30" t="inlineStr">
+        <is>
+          <t>s2_silver.fn_agg_fact_material_movements(snapshot_date)
+(+ by_postingdate variant for history)</t>
+        </is>
+      </c>
+      <c r="C4" s="30" t="inlineStr">
+        <is>
+          <t>Sum signed movement qty by stock type up to snapshot date; pivot stock types into columns; attach cost.</t>
+        </is>
+      </c>
+      <c r="D4" s="30" t="inlineStr">
+        <is>
+          <t>unrestricted_stock (01), stock_in_quality_inspection (02), blocked_*, stock_in_transit (06), total_stock_restricted_batches (08), ... + value columns</t>
+        </is>
+      </c>
+      <c r="E4" s="30" t="inlineStr">
+        <is>
+          <t>Physical stock portion of Inventory Units / Gross</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="85" customHeight="1" s="16">
+      <c r="A5" s="36" t="inlineStr">
+        <is>
+          <t>4. Gold snapshot union</t>
+        </is>
+      </c>
+      <c r="B5" s="30" t="inlineStr">
+        <is>
+          <t>eu_erp/s3_gold/nb_ebp_fact_inventory_snapshot_gold.ipynb
+→ s3_gold.fact_inventory_snapshot</t>
+        </is>
+      </c>
+      <c r="C5" s="30" t="inlineStr">
+        <is>
+          <t>UNION of MATDOC + ARUN allocated + STO + ATP into one daily snapshot grain.</t>
+        </is>
+      </c>
+      <c r="D5" s="30" t="inlineStr">
+        <is>
+          <t>Grain: snapshot_date, company_code, plant, material, storage_location, stock_segment, special_stock_indicator
+Metrics: unrestricted_use_stock, restricted_use_stock, allocated_to_*, sto_*, atp_wb_plant_stock, atp_la_shipping, atp_be_order_items, amt_*</t>
+        </is>
+      </c>
+      <c r="E5" s="30" t="inlineStr">
+        <is>
+          <t>Single backend fact before unpivot to cube</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="85" customHeight="1" s="16">
+      <c r="A6" s="36" t="inlineStr">
+        <is>
+          <t>5. Bridge unpivot for cube</t>
+        </is>
+      </c>
+      <c r="B6" s="30" t="inlineStr">
+        <is>
+          <t>s3_gold.fact_inventory_snapshot_bridge_eu</t>
+        </is>
+      </c>
+      <c r="C6" s="30" t="inlineStr">
+        <is>
+          <t>Unpivots metric columns into Inventory Type rows (QTYTYPE) and calculates Inventory Status / Gross / article &amp; DC keys.
+ATP_WB is exploded into -1 and +1 legs.</t>
+        </is>
+      </c>
+      <c r="D6" s="30" t="inlineStr">
+        <is>
+          <t>QTYTYPE, QTY, IntInventoryStatusCode, SPECIALSTOCKINDICATOR, STORAGELOCATION, STOCKSEGMENT, PLANT, MATERIAL, NatStoreDC_BK, NatArticle_BK, GROSS, POSTINGDATE, ArticleNumber_BK, ArticleSize_BK</t>
+        </is>
+      </c>
+      <c r="E6" s="30" t="inlineStr">
+        <is>
+          <t>Direct source of France DBX partition</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="85" customHeight="1" s="16">
+      <c r="A7" s="36" t="inlineStr">
+        <is>
+          <t>6. Assortment attributes</t>
+        </is>
+      </c>
+      <c r="B7" s="30" t="inlineStr">
+        <is>
+          <t>s3_gold.vw_inventory_material_assortment_semester</t>
+        </is>
+      </c>
+      <c r="C7" s="30" t="inlineStr">
+        <is>
+          <t>Provides First/Latest assortment semester per Material + CompanyCode (joined in France cube DBX partition).</t>
+        </is>
+      </c>
+      <c r="D7" s="30" t="inlineStr">
+        <is>
+          <t>MATERIAL, CompanyCode, FirstAssortment, LatestAssortment, PDUCode, IntPupMasterId</t>
+        </is>
+      </c>
+      <c r="E7" s="30" t="inlineStr">
+        <is>
+          <t>FirstAssortmentSemester / LatestAssortmentSemester → Actual/Old/Next/Discontinued</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="85" customHeight="1" s="16">
+      <c r="A8" s="36" t="inlineStr">
+        <is>
+          <t>7. Cube partition (France)</t>
+        </is>
+      </c>
+      <c r="B8" s="30" t="inlineStr">
+        <is>
+          <t>PDM - SUBS FRANCE - TEST INVENTORY
+fact_InventoryHistory / vFACT_InventoryHistory_DBX_FRA_CY</t>
+        </is>
+      </c>
+      <c r="C8" s="30" t="inlineStr">
+        <is>
+          <t>SELECT from bridge_eu where CompanyCode = FR10; maps DBX columns into cube table columns; SourceSystem = DBX.</t>
+        </is>
+      </c>
+      <c r="D8" s="30" t="inlineStr">
+        <is>
+          <t>Qty→InventoryUnits, QtyType→InventoryType, IntInventoryStatusCode→InventoryStatusCode, Gross→GrossValue, SpecialStockIndicator, StorageLocation, StockSegment, ...</t>
+        </is>
+      </c>
+      <c r="E8" s="30" t="inlineStr">
+        <is>
+          <t>All Inventory KPIs and dimension filters</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="85" customHeight="1" s="16">
+      <c r="A9" s="36" t="inlineStr">
+        <is>
+          <t>8. Cube measures (DAX)</t>
+        </is>
+      </c>
+      <c r="B9" s="30" t="inlineStr">
+        <is>
+          <t>Inventory Units, Total Free Inventory, Units Actual/Old/Next/Discontinued, Gross, ...</t>
+        </is>
+      </c>
+      <c r="C9" s="30" t="inlineStr">
+        <is>
+          <t>Front-end calculations on top of fact_InventoryHistory + calendar/assortment/status dimensions.</t>
+        </is>
+      </c>
+      <c r="D9" s="30" t="inlineStr">
+        <is>
+          <t>See KPIs List!Cube side Logic</t>
+        </is>
+      </c>
+      <c r="E9" s="30" t="inlineStr">
+        <is>
+          <t>What testers see in Power BI cards/matrices</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="70" customHeight="1" s="16">
+      <c r="A10" s="37" t="inlineStr">
+        <is>
+          <t>UAT note</t>
+        </is>
+      </c>
+      <c r="B10" s="37" t="inlineStr">
+        <is>
+          <t>Synapse path (SoT for parity)</t>
+        </is>
+      </c>
+      <c r="C10" s="37" t="inlineStr">
+        <is>
+          <t>Legacy path: staging movements → biz agg → etl.S4Hana_ProvInventories* → sourcing.InventoriesHistory via S4Hana_spProvInventories.
+Same conceptual grain, but DBX currently exposes more Allocated/ATP content and can include special stock E under UNRESTRICTEDSTOCK.</t>
+        </is>
+      </c>
+      <c r="D10" s="37" t="inlineStr">
+        <is>
+          <t>SPECIALSTOCKINDICATOR, QTYTYPE, IntInventoryStatusCode, Qty, StorageLocation, StockSegment</t>
+        </is>
+      </c>
+      <c r="E10" s="37" t="inlineStr">
+        <is>
+          <t>SourceSystem = EBP / OnPrem partitions in same France cube</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" style="16" min="1" max="1"/>
+    <col width="28" customWidth="1" style="16" min="2" max="2"/>
+    <col width="40" customWidth="1" style="16" min="3" max="3"/>
+    <col width="55" customWidth="1" style="16" min="4" max="4"/>
+    <col width="30" customWidth="1" style="16" min="5" max="5"/>
+    <col width="40" customWidth="1" style="16" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="35" customHeight="1" s="16">
+      <c r="A1" s="28" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="28" t="inlineStr">
+        <is>
+          <t>Cube column / filter</t>
+        </is>
+      </c>
+      <c r="C1" s="28" t="inlineStr">
+        <is>
+          <t>Databricks bridge / snapshot column</t>
+        </is>
+      </c>
+      <c r="D1" s="28" t="inlineStr">
+        <is>
+          <t>Backend logic (real DBX)</t>
+        </is>
+      </c>
+      <c r="E1" s="28" t="inlineStr">
+        <is>
+          <t>Used by KPI / dimension</t>
+        </is>
+      </c>
+      <c r="F1" s="28" t="inlineStr">
+        <is>
+          <t>Synapse vs DBX note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="95" customHeight="1" s="16">
+      <c r="A2" s="36" t="inlineStr">
+        <is>
+          <t>Inventory Units</t>
+        </is>
+      </c>
+      <c r="B2" s="37" t="inlineStr">
+        <is>
+          <t>bridge_eu.QTY
+(snapshot metric before unpivot: unrestricted_use_stock / allocated_* / sto_* / atp_*)</t>
+        </is>
+      </c>
+      <c r="C2" s="37" t="inlineStr">
+        <is>
+          <t>After STACK unpivot, each Inventory Type row carries its qty in QTY. Cube stores as InventoryUnits and measures SUM it with DAX filters.</t>
+        </is>
+      </c>
+      <c r="D2" s="37" t="inlineStr">
+        <is>
+          <t>Inventory Units and all Units* KPIs</t>
+        </is>
+      </c>
+      <c r="E2" s="37" t="inlineStr">
+        <is>
+          <t>DBX may include extra rows (Allocated, ATP, special stock E) under/near Unrestricted depending on filters.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="95" customHeight="1" s="16">
+      <c r="A3" s="36" t="inlineStr">
+        <is>
+          <t>Inventory Type</t>
+        </is>
+      </c>
+      <c r="B3" s="30" t="inlineStr">
+        <is>
+          <t>bridge_eu.QTYTYPE</t>
+        </is>
+      </c>
+      <c r="C3" s="30" t="inlineStr">
+        <is>
+          <t>Unpivot mapping:
+unrestricted_use_stock → UNRESTRICTEDSTOCK
+stock_in_quality_inspection → STOCKINQUALITYINSPECTION
+blocked_stock → BLOCKEDSTOCK
+stock_in_transit → STOCKINTRANSIT
+restricted_use_stock → TOTALSTOCKRESTRICTEDBATCHES
+allocated_to_stock/delivery/on_hold → ALLOCATED*
+sto_not_shipped/in_transit → STO*
+atp_wb/la/be also labeled UNRESTRICTEDSTOCK (different status)</t>
+        </is>
+      </c>
+      <c r="D3" s="30" t="inlineStr">
+        <is>
+          <t>Dimension: Inventory Type; main filter for Unrestricted tests</t>
+        </is>
+      </c>
+      <c r="E3" s="30" t="inlineStr">
+        <is>
+          <t>Allocated* mainly DBX-visible enrichment vs classic MATDOC-only compare.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="95" customHeight="1" s="16">
+      <c r="A4" s="36" t="inlineStr">
+        <is>
+          <t>Inventory Status / InventoryStatusCode</t>
+        </is>
+      </c>
+      <c r="B4" s="30" t="inlineStr">
+        <is>
+          <t>bridge_eu.IntInventoryStatusCode → dim_InventoryStatus</t>
+        </is>
+      </c>
+      <c r="C4" s="30" t="inlineStr">
+        <is>
+          <t>CASE logic in bridge_eu:
+ATP_WB ratio -1 → 10
+ATP_WB ratio +1 → 20
+ATP_BE → -20; ATP_LA → -10
+STO → 50
+special_stock_indicator = 'W' → 30
+stock_segment = 'CON' → 30
+plant category A (store) → 30
+ELSE → 10
+NOTE: special stock E currently falls into ELSE 10 (same as Unrestricted).</t>
+        </is>
+      </c>
+      <c r="D4" s="30" t="inlineStr">
+        <is>
+          <t>Dimension: Inventory Status; Free/Projected status</t>
+        </is>
+      </c>
+      <c r="E4" s="30" t="inlineStr">
+        <is>
+          <t>Same pattern as Synapse spProvInventories for W/CON/store; DBX adds ATP codes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="95" customHeight="1" s="16">
+      <c r="A5" s="36" t="inlineStr">
+        <is>
+          <t>Special Stock Indicator</t>
+        </is>
+      </c>
+      <c r="B5" s="37" t="inlineStr">
+        <is>
+          <t>bridge_eu.SPECIALSTOCKINDICATOR
+(= snapshot.special_stock_indicator ← movements.inventory_special_stock_type)</t>
+        </is>
+      </c>
+      <c r="C5" s="37" t="inlineStr">
+        <is>
+          <t>SAP SOBKZ. blank = normal own stock; W = consignment-like; E = customer/sales-order related special stock.
+Still counted in unrestricted_use_stock when MATDOC stock type = 01.</t>
+        </is>
+      </c>
+      <c r="D5" s="37" t="inlineStr">
+        <is>
+          <t>Dimension: Special Stock Indicator</t>
+        </is>
+      </c>
+      <c r="E5" s="37" t="inlineStr">
+        <is>
+          <t>CRITICAL: DBX Unrestricted includes E; Synapse SoT compare example matched blank only (3506 vs 6706).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="95" customHeight="1" s="16">
+      <c r="A6" s="36" t="inlineStr">
+        <is>
+          <t>Storage Location</t>
+        </is>
+      </c>
+      <c r="B6" s="30" t="inlineStr">
+        <is>
+          <t>bridge_eu.STORAGELOCATION</t>
+        </is>
+      </c>
+      <c r="C6" s="30" t="inlineStr">
+        <is>
+          <t>SAP LGORT. Part of snapshot grain. Example gap used 0001 (blank special stock) vs 0006 (E).</t>
+        </is>
+      </c>
+      <c r="D6" s="30" t="inlineStr">
+        <is>
+          <t>Dimension: Storage Location</t>
+        </is>
+      </c>
+      <c r="E6" s="30" t="inlineStr">
+        <is>
+          <t>Must be in UAT screenshots for deep dives.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="95" customHeight="1" s="16">
+      <c r="A7" s="36" t="inlineStr">
+        <is>
+          <t>Stock Segment</t>
+        </is>
+      </c>
+      <c r="B7" s="30" t="inlineStr">
+        <is>
+          <t>bridge_eu.STOCKSEGMENT</t>
+        </is>
+      </c>
+      <c r="C7" s="30" t="inlineStr">
+        <is>
+          <t>SAP segment (WHS/FRA/FPC/CON...). Used in NatStoreDC_BK (FR04_WHS|FR10). CON → status 30.</t>
+        </is>
+      </c>
+      <c r="D7" s="30" t="inlineStr">
+        <is>
+          <t>Dimension: Stock Segment; DC key</t>
+        </is>
+      </c>
+      <c r="E7" s="30" t="inlineStr">
+        <is>
+          <t>Confirm DC mapping when comparing FR04 vs FR04_WHS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="95" customHeight="1" s="16">
+      <c r="A8" s="36" t="inlineStr">
+        <is>
+          <t>Plant / Distribution Center</t>
+        </is>
+      </c>
+      <c r="B8" s="30" t="inlineStr">
+        <is>
+          <t>bridge_eu.PLANT + NatStoreDC_BK</t>
+        </is>
+      </c>
+      <c r="C8" s="30" t="inlineStr">
+        <is>
+          <t>NatStoreDC_BK = plant|company if store/empty segment, else plant_segment|company (PT10→ES10).</t>
+        </is>
+      </c>
+      <c r="D8" s="30" t="inlineStr">
+        <is>
+          <t>DC / plant filters in report</t>
+        </is>
+      </c>
+      <c r="E8" s="30" t="inlineStr">
+        <is>
+          <t>Compare using same NatStoreDC_BK, not only display name.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="95" customHeight="1" s="16">
+      <c r="A9" s="36" t="inlineStr">
+        <is>
+          <t>Material / Article / Size</t>
+        </is>
+      </c>
+      <c r="B9" s="30" t="inlineStr">
+        <is>
+          <t>MATERIAL, NatArticle_BK, ArticleNumber_BK, ArticleSize_BK</t>
+        </is>
+      </c>
+      <c r="C9" s="30" t="inlineStr">
+        <is>
+          <t>From dim_materials style/color/size. NatArticle = material|company.</t>
+        </is>
+      </c>
+      <c r="D9" s="30" t="inlineStr">
+        <is>
+          <t>Article filters; Torsten size-level checks</t>
+        </is>
+      </c>
+      <c r="E9" s="30" t="inlineStr">
+        <is>
+          <t>Watch typos (313502 vs 313504).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="95" customHeight="1" s="16">
+      <c r="A10" s="36" t="inlineStr">
+        <is>
+          <t>BookingDate</t>
+        </is>
+      </c>
+      <c r="B10" s="30" t="inlineStr">
+        <is>
+          <t>bridge_eu.POSTINGDATE (= snapshot_date for current snapshot bridge)</t>
+        </is>
+      </c>
+      <c r="C10" s="30" t="inlineStr">
+        <is>
+          <t>For current snapshot bridge, posting/booking date is the snapshot date. History/postingdate bridge keeps movement posting dates + running totals.</t>
+        </is>
+      </c>
+      <c r="D10" s="30" t="inlineStr">
+        <is>
+          <t>Calendar / current stock date context</t>
+        </is>
+      </c>
+      <c r="E10" s="30" t="inlineStr">
+        <is>
+          <t>For current stock use latest date; do not sum all dates of full balances.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="95" customHeight="1" s="16">
+      <c r="A11" s="36" t="inlineStr">
+        <is>
+          <t>Inventory Gross / GrossValue</t>
+        </is>
+      </c>
+      <c r="B11" s="30" t="inlineStr">
+        <is>
+          <t>bridge_eu.GROSS / VALUE; snapshot amt_*</t>
+        </is>
+      </c>
+      <c r="C11" s="30" t="inlineStr">
+        <is>
+          <t>PHYS/ALLOC/STO/ATP_LA/ATP_BE: GROSS from amount.
+ATP_WB gross forced to 0 in bridge CASE.
+Amount = qty * COALESCE(NULLIF(MAP,0), standard, 0) from dim_plant_material_cost.</t>
+        </is>
+      </c>
+      <c r="D11" s="30" t="inlineStr">
+        <is>
+          <t>Inventory Gross KPIs</t>
+        </is>
+      </c>
+      <c r="E11" s="30" t="inlineStr">
+        <is>
+          <t>Allocated rows can have Units but Gross 0 (UDPEBP-328). PRICECURRENCY blanks (UDPEBP-321).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="95" customHeight="1" s="16">
+      <c r="A12" s="36" t="inlineStr">
+        <is>
+          <t>First/Latest Assortment Semester</t>
+        </is>
+      </c>
+      <c r="B12" s="30" t="inlineStr">
+        <is>
+          <t>vw_inventory_material_assortment_semester.FirstAssortment / LatestAssortment
+(joined in France DBX partition on Material+CompanyCode)</t>
+        </is>
+      </c>
+      <c r="C12" s="30" t="inlineStr">
+        <is>
+          <t>From materialsalesattributes + company/interface. Used by DAX to split Actual/Old/Next/Discontinued.</t>
+        </is>
+      </c>
+      <c r="D12" s="30" t="inlineStr">
+        <is>
+          <t>Inventory Units Actual/Old/Next/Discontinued</t>
+        </is>
+      </c>
+      <c r="E12" s="30" t="inlineStr">
+        <is>
+          <t>If split differs but sum = Inventory Units → assortment mapping, not stock qty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="95" customHeight="1" s="16">
+      <c r="A13" s="36" t="inlineStr">
+        <is>
+          <t>SourceSystem</t>
+        </is>
+      </c>
+      <c r="B13" s="30" t="inlineStr">
+        <is>
+          <t>Literal 'DBX' in France DBX partitions; EBP/OnPrem from Synapse/on-prem partitions</t>
+        </is>
+      </c>
+      <c r="C13" s="30" t="inlineStr">
+        <is>
+          <t>Same cube table can contain multiple sources. Measures may combine them.</t>
+        </is>
+      </c>
+      <c r="D13" s="30" t="inlineStr">
+        <is>
+          <t>All KPIs</t>
+        </is>
+      </c>
+      <c r="E13" s="30" t="inlineStr">
+        <is>
+          <t>Always state SourceSystem when comparing SYN vs DBX.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="95" customHeight="1" s="16">
+      <c r="A14" s="36" t="inlineStr">
+        <is>
+          <t>Total Free Inventory (availability)</t>
+        </is>
+      </c>
+      <c r="B14" s="37" t="inlineStr">
+        <is>
+          <t>snapshot.atp_wb_plant_stock / atp_la_shipping / atp_be_order_items
+(+ free/available logic / projected status)</t>
+        </is>
+      </c>
+      <c r="C14" s="37" t="inlineStr">
+        <is>
+          <t>Not equal to MATDOC unrestricted.
+ATP_WB unpivoted as UNRESTRICTEDSTOCK with status 10 (-qty) and 20 (+qty).
+ATP_LA status -10, ATP_BE status -20.
+Business rule pending: deduct Allocated* from free or not.</t>
+        </is>
+      </c>
+      <c r="D14" s="37" t="inlineStr">
+        <is>
+          <t>Total Free Inventory / Inventory Status Projected</t>
+        </is>
+      </c>
+      <c r="E14" s="37" t="inlineStr">
+        <is>
+          <t>Main confusion point for Torsten + UDPEBP-323. Document filters before comparing.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -819,7 +1602,7 @@
       </c>
       <c r="G1" s="28" t="inlineStr">
         <is>
-          <t>Backend Logic (plain English)</t>
+          <t>Backend Logic (Databricks objects + plain English)</t>
         </is>
       </c>
       <c r="H1" s="28" t="inlineStr">
@@ -873,7 +1656,15 @@
       </c>
       <c r="G2" s="30" t="inlineStr">
         <is>
-          <t>Stock-on-hand quantity at material / plant / storage location / stock segment / batch / special stock.
+          <t>DBX path:
+1) s2_silver.fact_material_movements
+2) s2_silver.fn_agg_fact_material_movements(snapshot_date)
+3) s3_gold.fact_inventory_snapshot (MATDOC+ARUN+STO+ATP)
+4) s3_gold.fact_inventory_snapshot_bridge_eu → QTY
+5) Cube fact_InventoryHistory[InventoryUnits]
+Physical unrestricted column before unpivot: unrestricted_use_stock (MATDOC stock type 01).
+Cube Inventory Type filter uses QTYTYPE.
+Stock-on-hand quantity at material / plant / storage location / stock segment / batch / special stock.
 Source (DBX): s3_gold.fact_inventory_snapshot → bridge view fact_inventory_snapshot_bridge_eu.
 Physical stock comes from SAP MATDOC movements (stock type 01/02/03/... mapped to Inventory Type).
 Cube field: InventoryUnits = Qty from bridge.
@@ -931,7 +1722,11 @@
       </c>
       <c r="G3" s="30" t="inlineStr">
         <is>
-          <t>Business name for 'free / available' inventory (Torsten referred to this as free inventory units).
+          <t>DBX path:
+s3_gold.fact_inventory_snapshot.atp_wb_plant_stock / atp_la_shipping / atp_be_order_items
+(+ allocation columns allocated_to_*), exposed via bridge_eu with Inventory Status codes 10/20/-10/-20.
+Not the same as unrestricted_use_stock only.
+Business name for 'free / available' inventory (Torsten referred to this as free inventory units).
 In DBX this is NOT pure MATDOC unrestricted.
 It is built from inventory snapshot plus availability logic (ATP / free-to-allocate concepts):
 - Plant stock (WB)
@@ -1011,7 +1806,15 @@
       </c>
       <c r="G4" s="30" t="inlineStr">
         <is>
-          <t>Subset of Inventory Units for articles that are in an active assortment for the selected semester.
+          <t>DBX path:
+1) s2_silver.fact_material_movements
+2) s2_silver.fn_agg_fact_material_movements(snapshot_date)
+3) s3_gold.fact_inventory_snapshot (MATDOC+ARUN+STO+ATP)
+4) s3_gold.fact_inventory_snapshot_bridge_eu → QTY
+5) Cube fact_InventoryHistory[InventoryUnits]
+Physical unrestricted column before unpivot: unrestricted_use_stock (MATDOC stock type 01).
+Cube Inventory Type filter uses QTYTYPE.
+Subset of Inventory Units for articles that are in an active assortment for the selected semester.
 Backend fields used: FirstAssortmentSemester and LatestAssortmentSemester (from assortment / material sales attributes).
 Rule: FirstAssortmentSemester &lt;= selected semester &lt;= LatestAssortmentSemester.</t>
         </is>
@@ -1107,7 +1910,15 @@
       </c>
       <c r="G5" s="30" t="inlineStr">
         <is>
-          <t>Inventory of articles whose latest assortment semester is older than the selected semester (old/previous assortment).
+          <t>DBX path:
+1) s2_silver.fact_material_movements
+2) s2_silver.fn_agg_fact_material_movements(snapshot_date)
+3) s3_gold.fact_inventory_snapshot (MATDOC+ARUN+STO+ATP)
+4) s3_gold.fact_inventory_snapshot_bridge_eu → QTY
+5) Cube fact_InventoryHistory[InventoryUnits]
+Physical unrestricted column before unpivot: unrestricted_use_stock (MATDOC stock type 01).
+Cube Inventory Type filter uses QTYTYPE.
+Inventory of articles whose latest assortment semester is older than the selected semester (old/previous assortment).
 Uses LatestAssortmentSemester vs selected semester (semester number / season logic).</t>
         </is>
       </c>
@@ -1176,7 +1987,15 @@
       </c>
       <c r="G6" s="30" t="inlineStr">
         <is>
-          <t>Inventory of articles whose first assortment semester is after the selected semester (future assortment / not yet active).</t>
+          <t>DBX path:
+1) s2_silver.fact_material_movements
+2) s2_silver.fn_agg_fact_material_movements(snapshot_date)
+3) s3_gold.fact_inventory_snapshot (MATDOC+ARUN+STO+ATP)
+4) s3_gold.fact_inventory_snapshot_bridge_eu → QTY
+5) Cube fact_InventoryHistory[InventoryUnits]
+Physical unrestricted column before unpivot: unrestricted_use_stock (MATDOC stock type 01).
+Cube Inventory Type filter uses QTYTYPE.
+Inventory of articles whose first assortment semester is after the selected semester (future assortment / not yet active).</t>
         </is>
       </c>
       <c r="H6" s="30" t="inlineStr">
@@ -1268,7 +2087,15 @@
       </c>
       <c r="G7" s="30" t="inlineStr">
         <is>
-          <t>Inventory of articles discontinued relative to selected semester (latest assortment just before current semester – discontinued bucket).</t>
+          <t>DBX path:
+1) s2_silver.fact_material_movements
+2) s2_silver.fn_agg_fact_material_movements(snapshot_date)
+3) s3_gold.fact_inventory_snapshot (MATDOC+ARUN+STO+ATP)
+4) s3_gold.fact_inventory_snapshot_bridge_eu → QTY
+5) Cube fact_InventoryHistory[InventoryUnits]
+Physical unrestricted column before unpivot: unrestricted_use_stock (MATDOC stock type 01).
+Cube Inventory Type filter uses QTYTYPE.
+Inventory of articles discontinued relative to selected semester (latest assortment just before current semester – discontinued bucket).</t>
         </is>
       </c>
       <c r="H7" s="30" t="inlineStr">
@@ -1325,7 +2152,15 @@
       </c>
       <c r="G8" s="30" t="inlineStr">
         <is>
-          <t>Same Inventory Units logic shifted to same period last year (time-intelligence).</t>
+          <t>DBX path:
+1) s2_silver.fact_material_movements
+2) s2_silver.fn_agg_fact_material_movements(snapshot_date)
+3) s3_gold.fact_inventory_snapshot (MATDOC+ARUN+STO+ATP)
+4) s3_gold.fact_inventory_snapshot_bridge_eu → QTY
+5) Cube fact_InventoryHistory[InventoryUnits]
+Physical unrestricted column before unpivot: unrestricted_use_stock (MATDOC stock type 01).
+Cube Inventory Type filter uses QTYTYPE.
+Same Inventory Units logic shifted to same period last year (time-intelligence).</t>
         </is>
       </c>
       <c r="H8" s="30" t="inlineStr">
@@ -1366,7 +2201,15 @@
       </c>
       <c r="G9" s="30" t="inlineStr">
         <is>
-          <t>Difference: current Inventory Units Comp − Inventory Units LY.</t>
+          <t>DBX path:
+1) s2_silver.fact_material_movements
+2) s2_silver.fn_agg_fact_material_movements(snapshot_date)
+3) s3_gold.fact_inventory_snapshot (MATDOC+ARUN+STO+ATP)
+4) s3_gold.fact_inventory_snapshot_bridge_eu → QTY
+5) Cube fact_InventoryHistory[InventoryUnits]
+Physical unrestricted column before unpivot: unrestricted_use_stock (MATDOC stock type 01).
+Cube Inventory Type filter uses QTYTYPE.
+Difference: current Inventory Units Comp − Inventory Units LY.</t>
         </is>
       </c>
       <c r="H9" s="30" t="inlineStr">
@@ -1407,7 +2250,15 @@
       </c>
       <c r="G10" s="30" t="inlineStr">
         <is>
-          <t>Percentage variance vs last year = (Units vs LY) / abs(Units LY).</t>
+          <t>DBX path:
+1) s2_silver.fact_material_movements
+2) s2_silver.fn_agg_fact_material_movements(snapshot_date)
+3) s3_gold.fact_inventory_snapshot (MATDOC+ARUN+STO+ATP)
+4) s3_gold.fact_inventory_snapshot_bridge_eu → QTY
+5) Cube fact_InventoryHistory[InventoryUnits]
+Physical unrestricted column before unpivot: unrestricted_use_stock (MATDOC stock type 01).
+Cube Inventory Type filter uses QTYTYPE.
+Percentage variance vs last year = (Units vs LY) / abs(Units LY).</t>
         </is>
       </c>
       <c r="H10" s="30" t="inlineStr">
@@ -1459,7 +2310,10 @@
       </c>
       <c r="G11" s="30" t="inlineStr">
         <is>
-          <t>Inventory value (amount), not units.
+          <t>DBX: snapshot amt_* and bridge GROSS/VALUE
+Price from s3_gold.dim_plant_material_cost (MAP else standard).
+Allocated Gross may be 0 even when Units &gt; 0.
+Inventory value (amount), not units.
 Backend: quantity × cost (moving average price if available, else standard price) from plant/material cost.
 Cube can show LC or converted EUR via FX.</t>
         </is>
@@ -1516,7 +2370,10 @@
       </c>
       <c r="G12" s="30" t="inlineStr">
         <is>
-          <t>Inventory Gross for same period last year.</t>
+          <t>DBX: snapshot amt_* and bridge GROSS/VALUE
+Price from s3_gold.dim_plant_material_cost (MAP else standard).
+Allocated Gross may be 0 even when Units &gt; 0.
+Inventory Gross for same period last year.</t>
         </is>
       </c>
       <c r="H12" s="30" t="inlineStr">
@@ -1558,7 +2415,10 @@
       </c>
       <c r="G13" s="30" t="inlineStr">
         <is>
-          <t>Inventory Gross − Inventory Gross LY.</t>
+          <t>DBX: snapshot amt_* and bridge GROSS/VALUE
+Price from s3_gold.dim_plant_material_cost (MAP else standard).
+Allocated Gross may be 0 even when Units &gt; 0.
+Inventory Gross − Inventory Gross LY.</t>
         </is>
       </c>
       <c r="H13" s="30" t="inlineStr">
@@ -1599,7 +2459,10 @@
       </c>
       <c r="G14" s="30" t="inlineStr">
         <is>
-          <t>(Gross vs LY) / abs(Gross LY).</t>
+          <t>DBX: snapshot amt_* and bridge GROSS/VALUE
+Price from s3_gold.dim_plant_material_cost (MAP else standard).
+Allocated Gross may be 0 even when Units &gt; 0.
+(Gross vs LY) / abs(Gross LY).</t>
         </is>
       </c>
       <c r="H14" s="30" t="inlineStr">
@@ -1647,7 +2510,15 @@
       </c>
       <c r="G15" s="30" t="inlineStr">
         <is>
-          <t>Inventory Units aligned to Delivery Date dimension instead of normal calendar/booking date.
+          <t>DBX path:
+1) s2_silver.fact_material_movements
+2) s2_silver.fn_agg_fact_material_movements(snapshot_date)
+3) s3_gold.fact_inventory_snapshot (MATDOC+ARUN+STO+ATP)
+4) s3_gold.fact_inventory_snapshot_bridge_eu → QTY
+5) Cube fact_InventoryHistory[InventoryUnits]
+Physical unrestricted column before unpivot: unrestricted_use_stock (MATDOC stock type 01).
+Cube Inventory Type filter uses QTYTYPE.
+Inventory Units aligned to Delivery Date dimension instead of normal calendar/booking date.
 Uses bookings by delivery date + Databricks bookings component.</t>
         </is>
       </c>
@@ -1692,7 +2563,15 @@
       </c>
       <c r="G16" s="30" t="inlineStr">
         <is>
-          <t>Same as Delivery Date Units, but using BookingDateLW relationship (last-week style shift).</t>
+          <t>DBX path:
+1) s2_silver.fact_material_movements
+2) s2_silver.fn_agg_fact_material_movements(snapshot_date)
+3) s3_gold.fact_inventory_snapshot (MATDOC+ARUN+STO+ATP)
+4) s3_gold.fact_inventory_snapshot_bridge_eu → QTY
+5) Cube fact_InventoryHistory[InventoryUnits]
+Physical unrestricted column before unpivot: unrestricted_use_stock (MATDOC stock type 01).
+Cube Inventory Type filter uses QTYTYPE.
+Same as Delivery Date Units, but using BookingDateLW relationship (last-week style shift).</t>
         </is>
       </c>
       <c r="H16" s="30" t="inlineStr">
@@ -1730,7 +2609,9 @@
       <c r="F17" s="34" t="n"/>
       <c r="G17" s="34" t="inlineStr">
         <is>
-          <t>Technical field QTYTYPE from backend bridge.
+          <t>DBX column: fact_inventory_snapshot_bridge_eu.QTYTYPE
+Created by STACK() over snapshot metrics in bridge_eu SQL.
+Technical field QTYTYPE from backend bridge.
 Main values:
 - UNRESTRICTEDSTOCK (MATDOC stock type 01)
 - STOCKINQUALITYINSPECTION (02)
@@ -1857,7 +2738,13 @@
       <c r="F20" s="34" t="n"/>
       <c r="G20" s="34" t="inlineStr">
         <is>
-          <t>SAP special stock indicator (SOBKZ).
+          <t>DBX columns:
+fact_material_movements.inventory_special_stock_type
+→ fact_inventory_snapshot.special_stock_indicator
+→ bridge_eu.SPECIALSTOCKINDICATOR
+→ cube SpecialStockIndicator.
+Status mapping in bridge only special-cases 'W' today; 'E' currently status 10.
+SAP special stock indicator (SOBKZ).
 - blank = normal own stock
 - W = consignment / reserved-like (status 30)
 - E = customer / sales-order related special stock (customer-owned/allocated style stock)
@@ -1904,7 +2791,9 @@
       <c r="F21" s="34" t="n"/>
       <c r="G21" s="34" t="inlineStr">
         <is>
-          <t>Mapped from IntInventoryStatusCode in bridge/provisioning:
+          <t>DBX column: bridge_eu.IntInventoryStatusCode
+Logic in fact_inventory_snapshot_bridge_eu CASE expression (ATP/STO/W/CON/store/else).
+Mapped from IntInventoryStatusCode in bridge/provisioning:
 - 10 = normal / unrestricted-like
 - 20 = ATP WB credit side / allocated-like projection
 - 30 = reserved-like (special stock W, CON segment, store plant category A)
@@ -1950,7 +2839,9 @@
       <c r="F22" s="34" t="n"/>
       <c r="G22" s="34" t="inlineStr">
         <is>
-          <t>Status used for projected / free / ATP inventory views.
+          <t>DBX column: bridge_eu.IntInventoryStatusCode
+Logic in fact_inventory_snapshot_bridge_eu CASE expression (ATP/STO/W/CON/store/else).
+Status used for projected / free / ATP inventory views.
 Separates physical stock from projected availability components.</t>
         </is>
       </c>
@@ -2030,13 +2921,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18.7109375" customWidth="1" style="3" min="1" max="1"/>
@@ -2475,7 +3366,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Rewrite inventory testing workbook in working notes style
Keep DBX backend flow/logic in one column, Synapse vs DBX in another,
drop How-to-test and Torsten/meta guidance so the sheet reads like
normal UAT documentation.

Co-authored-by: Akshay97 <axayteja_de@hotmail.com>
</commit_message>
<xml_diff>
--- a/Inventory_Testing.xlsx
+++ b/Inventory_Testing.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,8 +28,14 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="4">
@@ -46,7 +52,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -60,35 +66,31 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00B0B0B0"/>
+        <color rgb="00D9D9D9"/>
       </left>
       <right style="thin">
-        <color rgb="00B0B0B0"/>
+        <color rgb="00D9D9D9"/>
       </right>
       <top style="thin">
-        <color rgb="00B0B0B0"/>
+        <color rgb="00D9D9D9"/>
       </top>
       <bottom style="thin">
-        <color rgb="00B0B0B0"/>
+        <color rgb="00D9D9D9"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -461,15 +463,15 @@
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
-    <col width="58" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>No</t>
@@ -511,7 +513,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="105" customHeight="1">
+    <row r="2" ht="110" customHeight="1">
       <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
@@ -554,73 +556,72 @@
 s2_silver.fact_material_movements
 → s2_silver.fn_agg_fact_material_movements(snapshot_date)
 → s3_gold.fact_inventory_snapshot
-→ s3_gold.fact_inventory_snapshot_bridge_eu (QTY)
+→ s3_gold.fact_inventory_snapshot_bridge_eu (QTY / QTYTYPE)
 → cube fact_InventoryHistory[InventoryUnits]
 Logic:
-- Physical stock = cumulative signed MATDOC qty by inventory_stock_type
+- physical stock = cumulative signed MATDOC qty by inventory_stock_type
 - unrestricted_use_stock = stock type 01
-- Snapshot also unions ARUN allocated, STO and ATP
-- Bridge unpivots metrics to QTYTYPE; cube sums QTY
-- Grain: plant, material, storage_location, stock_segment, special_stock_indicator, batch</t>
+- snapshot also brings in ARUN allocated, STO and ATP
+- bridge unpivots the qty metrics into QTYTYPE, cube just sums QTY
+- grain: plant, material, storage_location, stock_segment, special_stock_indicator, batch</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Synapse is the parity reference.
-DBX can show higher Unrestricted when special stock E is included, and also has Allocated/ATP rows.
-Checked example: 026404-01-150 / FR04 / UNRESTRICTEDSTOCK → Synapse 3,506; DBX 6,706 (= 3,506 blank special stock + 3,200 special stock E at 0006).</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="105" customHeight="1">
-      <c r="A3" s="2" t="n">
+          <t>For Unrestricted, DBX can come higher than Synapse because special stock E is still inside UNRESTRICTEDSTOCK.
+Example we checked: 026404-01-150 / FR04 / UNRESTRICTEDSTOCK → Syn 3,506 | DBX 6,706 (3,506 blank special stock + 3,200 E at LGORT 0006).
+Allocated / ATP rows are also more visible on DBX.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="110" customHeight="1">
+      <c r="A3" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>KPI</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>Inventory Units Projected</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Total Free Inventory</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>In-Progress</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="n"/>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>In-Progress</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="n"/>
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Flow:
 s3_gold.fact_inventory_snapshot
-- unrestricted_use_stock
-- allocated_to_stock / allocated_to_delivery / allocated_on_hold
-- atp_wb_plant_stock / atp_la_shipping / atp_be_order_items
-→ bridge_eu (mostly QTYTYPE=UNRESTRICTEDSTOCK with different IntInventoryStatusCode)
+  unrestricted_use_stock
+  allocated_to_stock / allocated_to_delivery / allocated_on_hold
+  atp_wb_plant_stock / atp_la_shipping / atp_be_order_items
+→ bridge_eu (ATP mostly still under QTYTYPE = UNRESTRICTEDSTOCK, status differs)
 → cube Total Free Inventory / projected measures
 Logic:
-- Not the same as pure MATDOC unrestricted
-- ATP_WB → status 10 (-qty) and 20 (+qty)
+- this is not pure MATDOC unrestricted
+- ATP_WB → status 10 (-qty) / 20 (+qty)
 - ATP_LA → -10, ATP_BE → -20
-- Open point: whether Allocated should be deducted here like legacy free logic</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Mismatch under UDPEBP-323.
-DBX ATP breakout is more explicit than what we usually validated in Synapse.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="105" customHeight="1">
+- still open whether Allocated should be deducted here like the old free logic</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Mismatch logged under UDPEBP-323. DBX shows ATP components more clearly than what we usually had on Synapse.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="110" customHeight="1">
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
@@ -677,44 +678,44 @@
       <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Flow:
-bridge_eu inventory qty
+bridge_eu qty
 + s3_gold.vw_inventory_material_assortment_semester
   (France DBX partition join on Material + CompanyCode)
 → FirstAssortmentSemester / LatestAssortmentSemester
 → DAX Actual bucket
 Logic:
-Actual when selected semester is between First and Latest assortment semester.
+Actual when selected semester sits between First and Latest assortment semester.
 OnPrem path uses IntAgeingCode = 20.</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>SYN vs DBX split can differ if assortment semesters differ.
-If Actual+Old+Next+Discontinued still equal Inventory Units, qty is fine and assortment mapping needs check (UDPEBP-324).</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="105" customHeight="1">
-      <c r="A5" s="2" t="n">
+          <t>Split can differ SYN vs DBX if assortment semester values differ.
+If Actual+Old+Next+Discontinued still equals Inventory Units, qty is fine and issue is assortment mapping (UDPEBP-324).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="70" customHeight="1">
+      <c r="A5" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>KPI</t>
         </is>
       </c>
-      <c r="C5" s="2" t="n"/>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="C5" s="3" t="n"/>
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>Inventory Units Old</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>In-Progress</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>In-Progress</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>VAR SelectedSemesterNumber =
     MAX ( 'dim_Calendar'[SemesterNumber] )
@@ -769,20 +770,20 @@
     )</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>Same qty flow as Inventory Units.
-Bucketed when LatestAssortmentSemester is older than selected semester.
+Goes to Old when LatestAssortmentSemester is older than selected semester.
 OnPrem path uses IntAgeingCode = 40.</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>Usually assortment-split difference, not MATDOC qty difference.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="105" customHeight="1">
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Usually assortment split difference, not MATDOC qty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="70" customHeight="1">
       <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
@@ -837,37 +838,37 @@
       <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Same qty flow as Inventory Units.
-Bucketed when FirstAssortmentSemester &gt; selected semester.
+Goes to Next when FirstAssortmentSemester &gt; selected semester.
 OnPrem path uses IntAgeingCode = 10.</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Check FirstAssortmentSemester in DBX vs Synapse.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="105" customHeight="1">
-      <c r="A7" s="2" t="n">
+          <t>Check FirstAssortmentSemester population in DBX vs Synapse.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="70" customHeight="1">
+      <c r="A7" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>KPI</t>
         </is>
       </c>
-      <c r="C7" s="2" t="n"/>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="C7" s="3" t="n"/>
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>inventory Units Discontinued</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>In-Progress</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>In-Progress</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">VAR SelectedSemesterNumber =
     MAX ( 'dim_Calendar'[SemesterNumber] )
@@ -923,20 +924,20 @@
     </t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>Same qty flow as Inventory Units.
-Bucketed as discontinued vs selected semester using LatestAssortmentSemester offset logic.
+Discontinued bucket uses LatestAssortmentSemester offset vs selected semester.
 OnPrem path uses IntAgeingCode = 30.</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>Reconcile with Actual/Old/Next against Inventory Units total.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="105" customHeight="1">
+    <row r="8" ht="70" customHeight="1">
       <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
@@ -979,54 +980,53 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Same DBX inventory fact/bridge qty.
-Cube applies last-year timing via LY measure logic.</t>
+          <t>Same inventory fact/bridge qty from DBX.
+LY shift is done in the cube measure.</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Values looked as expected in current tests.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="105" customHeight="1">
-      <c r="A9" s="2" t="n">
+          <t>Values looked fine in current tests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="70" customHeight="1">
+      <c r="A9" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>KPI</t>
         </is>
       </c>
-      <c r="C9" s="2" t="n"/>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="C9" s="3" t="n"/>
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>inventory units vs LY</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>In-Progress</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>In-Progress</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>[Inventory Units Comp] - [Inventory Units LY]</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>Derived in cube from current units and units LY.
-No separate backend metric.</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>Follows Units and Units LY.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="105" customHeight="1">
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Cube calc only: current units − units LY. No separate backend metric.</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Depends on Units and Units LY.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="70" customHeight="1">
       <c r="A10" s="2" t="n">
         <v>9</v>
       </c>
@@ -1053,37 +1053,36 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Derived % in cube.
-No separate backend metric.</t>
+          <t>Cube calc only: Units vs LY / abs(Units LY). No separate backend metric.</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Follows Units and Units LY.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="105" customHeight="1">
-      <c r="A11" s="2" t="n">
+          <t>Depends on Units and Units LY.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="110" customHeight="1">
+      <c r="A11" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>KPI</t>
         </is>
       </c>
-      <c r="C11" s="2" t="n"/>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="C11" s="3" t="n"/>
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>Inventory Gross</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>In-Progress</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>In-Progress</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>VAR IsEURSel = [FXSelect] = "EUR"
 RETURN
@@ -1099,7 +1098,7 @@
     )</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>Flow:
 snapshot qty
@@ -1109,19 +1108,19 @@
 → cube Inventory Gross
 Logic:
 - GROSS kept for PHYS / ALLOC / STO / ATP_LA / ATP_BE
-- ATP_WB gross = 0 in bridge
-- Missing cost ⇒ units can exist with gross 0</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>UDPEBP-325 aggregated Gross display in DBX.
-UDPEBP-328 Allocated Units without Gross.
-UDPEBP-321 PRICECURRENCY blanks.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="105" customHeight="1">
+- ATP_WB gross forced to 0 in bridge
+- if cost is missing, units can still show with gross 0</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>UDPEBP-325: aggregated Gross not showing properly in DBX.
+UDPEBP-328: Allocated units without Gross.
+UDPEBP-321: PRICECURRENCY blanks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="70" customHeight="1">
       <c r="A12" s="2" t="n">
         <v>11</v>
       </c>
@@ -1159,7 +1158,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Same gross backend as Inventory Gross; cube applies LY timing/FX.</t>
+          <t>Same gross backend as Inventory Gross; LY / FX handled in cube.</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1168,44 +1167,44 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="105" customHeight="1">
-      <c r="A13" s="2" t="n">
+    <row r="13" ht="70" customHeight="1">
+      <c r="A13" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>KPI</t>
         </is>
       </c>
-      <c r="C13" s="2" t="n"/>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="C13" s="3" t="n"/>
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t>Inventory Gross Vs LY</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>In-Progress</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>In-Progress</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>--[Inventory Gross Comp] 
 [Inventory Gross]- [Inventory Gross LY]</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>Derived in cube. No separate backend metric.</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Cube calc only: Gross − Gross LY. No separate backend metric.</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
         <is>
           <t>Depends on Gross and Gross LY.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="105" customHeight="1">
+    <row r="14" ht="70" customHeight="1">
       <c r="A14" s="2" t="n">
         <v>13</v>
       </c>
@@ -1232,7 +1231,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Derived in cube. No separate backend metric.</t>
+          <t>Cube calc only: Gross vs LY / abs(Gross LY). No separate backend metric.</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1241,27 +1240,27 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="105" customHeight="1">
-      <c r="A15" s="2" t="n">
+    <row r="15" ht="70" customHeight="1">
+      <c r="A15" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>KPI</t>
         </is>
       </c>
-      <c r="C15" s="2" t="n"/>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="C15" s="3" t="n"/>
+      <c r="D15" s="3" t="inlineStr">
         <is>
           <t>Inventory Units Delivery Date</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>In-Progress</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>In-Progress</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>/* ToDo: DAX Optimizing */
 VAR LastCubeProcDate = [Last Cube Processing Date]
@@ -1273,19 +1272,19 @@
     )</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G15" s="3" t="inlineStr">
         <is>
           <t>Same inventory qty from snapshot/bridge.
-Cube evaluates against Delivery Date dimension and bookings components.</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>UDPEBP-326: differs when Delivery Date is used.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="105" customHeight="1">
+Cube evaluates it against Delivery Date + bookings side.</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>UDPEBP-326: values differ when Delivery Date is used.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="70" customHeight="1">
       <c r="A16" s="2" t="n">
         <v>15</v>
       </c>
@@ -1325,7 +1324,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="105" customHeight="1">
+    <row r="17" ht="110" customHeight="1">
       <c r="A17" s="3" t="n">
         <v>16</v>
       </c>
@@ -1352,8 +1351,8 @@
       <c r="F17" s="3" t="n"/>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>DBX column: fact_inventory_snapshot_bridge_eu.QTYTYPE
-Cube column: InventoryType
+          <t>DBX: fact_inventory_snapshot_bridge_eu.QTYTYPE
+Cube: InventoryType
 Unpivot:
 - unrestricted_use_stock → UNRESTRICTEDSTOCK
 - QI / blocked / transit / restricted → matching type names
@@ -1364,51 +1363,50 @@
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>DBX shows Allocated* more explicitly.
-For MATDOC compares we filter UNRESTRICTEDSTOCK and also check special stock/status.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="105" customHeight="1">
-      <c r="A18" s="3" t="n">
+          <t>DBX exposes Allocated* more clearly.
+For MATDOC compares we filter UNRESTRICTEDSTOCK and also look at special stock / status.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="70" customHeight="1">
+      <c r="A18" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>Dimension</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>Inventory Details</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>Stock Segment</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>In-Progress</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="n"/>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t>DBX: bridge_eu.STOCKSEGMENT ← snapshot.stock_segment
-From movements segment fields.
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>In-Progress</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="n"/>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>DBX: bridge_eu.STOCKSEGMENT ← snapshot.stock_segment (from movements).
 Used in NatStoreDC_BK (e.g. FR04_WHS|FR10).
-CON → status 30.</t>
-        </is>
-      </c>
-      <c r="H18" s="3" t="inlineStr">
-        <is>
-          <t>Generally aligned; watch model-specific segment exclusions like FPC.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="105" customHeight="1">
+CON → Inventory Status 30.</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Mostly aligned. Watch model-specific exclusions like FPC if used.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="70" customHeight="1">
       <c r="A19" s="3" t="n">
         <v>18</v>
       </c>
@@ -1435,44 +1433,44 @@
       <c r="F19" s="3" t="n"/>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>DBX: bridge_eu.STORAGELOCATION ← snapshot.storage_location (SAP LGORT)
-Part of grain with plant/material/segment/special stock.</t>
+          <t>DBX: bridge_eu.STORAGELOCATION ← snapshot.storage_location (SAP LGORT).
+Part of grain with plant / material / segment / special stock.</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>Useful for gaps like 0001 vs 0006 in the special stock E case.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="105" customHeight="1">
-      <c r="A20" s="3" t="n">
+          <t>Helps explain gaps like 0001 vs 0006 in the special stock E case.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="110" customHeight="1">
+      <c r="A20" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>Dimension</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>Inventory Details</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>Special Stock Indicator</t>
         </is>
       </c>
-      <c r="E20" s="3" t="inlineStr">
-        <is>
-          <t>In-Progress</t>
-        </is>
-      </c>
-      <c r="F20" s="3" t="n"/>
-      <c r="G20" s="3" t="inlineStr">
-        <is>
-          <t>DBX flow:
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>In-Progress</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="n"/>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Flow:
 fact_material_movements.inventory_special_stock_type
 → fact_inventory_snapshot.special_stock_indicator
 → bridge_eu.SPECIALSTOCKINDICATOR
@@ -1480,20 +1478,20 @@
 Logic:
 - blank = normal own stock
 - W → Inventory Status 30
-- E currently not specially mapped, so stays status 10 and can remain under UNRESTRICTEDSTOCK when stock type = 01
-- E is customer/sales-order related stock
-- For parity we treat Synapse as SoT and need to align Unrestricted handling of E</t>
-        </is>
-      </c>
-      <c r="H20" s="3" t="inlineStr">
-        <is>
-          <t>Main current Unrestricted gap.
+- E is not specially mapped today → stays status 10 and can remain under UNRESTRICTEDSTOCK when stock type = 01
+- E is customer / sales-order related stock
+- for Synapse parity we need to decide how Unrestricted should treat E</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>This is the main Unrestricted gap right now.
 Synapse SP keeps SPECIALSTOCKINDICATOR and only forces W→30; E is not explicitly dropped there.
-In compared totals, Synapse matched blank-special-stock qty only.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="105" customHeight="1">
+In the compared totals though, Synapse matched the blank-special-stock qty only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="110" customHeight="1">
       <c r="A21" s="3" t="n">
         <v>20</v>
       </c>
@@ -1536,45 +1534,45 @@
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>DBX ATP statuses are more visible.
-Inventory Type = UNRESTRICTEDSTOCK alone can still include ATP rows.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="105" customHeight="1">
-      <c r="A22" s="3" t="n">
+          <t>ATP statuses show up more on DBX.
+Filtering Inventory Type = UNRESTRICTEDSTOCK alone can still include ATP rows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="70" customHeight="1">
+      <c r="A22" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>Dimension</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>Inventory Status</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>Inventory Status Projected</t>
         </is>
       </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>In-Progress</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="n"/>
-      <c r="G22" s="3" t="inlineStr">
-        <is>
-          <t>Used for projected/free availability.
-Backed by same IntInventoryStatusCode / ATP columns from snapshot + bridge_eu.</t>
-        </is>
-      </c>
-      <c r="H22" s="3" t="inlineStr">
-        <is>
-          <t>More relevant in DBX because ATP components are richer.</t>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>In-Progress</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="n"/>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Used for projected / free availability.
+Same IntInventoryStatusCode / ATP columns from snapshot + bridge_eu.</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>More relevant on DBX because ATP components are richer.</t>
         </is>
       </c>
     </row>
@@ -1592,29 +1590,29 @@
   <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Cube field</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>DBX object.column</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Logic</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="40" customHeight="1">
+    <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>InventoryUnits</t>
@@ -1627,28 +1625,28 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Unpivoted qty from snapshot metrics; summed by cube measures.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="40" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
+          <t>Unpivoted qty from snapshot metrics; cube measures sum this.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>InventoryType</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>bridge_eu.QTYTYPE</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>STACK unpivot of unrestricted/allocated/sto/restricted/etc. ATP currently also uses UNRESTRICTEDSTOCK.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="40" customHeight="1">
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>STACK unpivot of unrestricted / allocated / sto / restricted / etc. ATP currently also under UNRESTRICTEDSTOCK.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>InventoryStatusCode</t>
@@ -1661,28 +1659,28 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>CASE on ATP/STO/special stock W/CON/store/else. Description via dim_InventoryStatus.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="40" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
+          <t>CASE on ATP / STO / special stock W / CON / store / else. Description comes from dim_InventoryStatus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>SpecialStockIndicator</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>bridge_eu.SPECIALSTOCKINDICATOR</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>From movements.inventory_special_stock_type → snapshot.special_stock_indicator.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="40" customHeight="1">
+    <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>StorageLocation</t>
@@ -1699,24 +1697,24 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="40" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>StockSegment</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>bridge_eu.STOCKSEGMENT</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>SAP segment; used in NatStoreDC_BK.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="40" customHeight="1">
+    <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Plant</t>
@@ -1729,28 +1727,28 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>SAP plant/DC.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="40" customHeight="1">
-      <c r="A9" s="2" t="inlineStr">
+          <t>SAP plant / DC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Material / Article fields</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>MATERIAL / NatArticle_BK / ArticleNumber_BK / ArticleSize_BK</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>Material plus dim_materials article attributes.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="40" customHeight="1">
+    <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>BookingDate</t>
@@ -1767,24 +1765,24 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="40" customHeight="1">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>GrossValue</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>bridge_eu.GROSS / VALUE (+ snapshot amt_*)</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Qty x cost from dim_plant_material_cost; ATP_WB gross = 0.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="40" customHeight="1">
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Qty × cost from dim_plant_material_cost; ATP_WB gross = 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
           <t>First/Latest Assortment Semester</t>
@@ -1801,20 +1799,20 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="40" customHeight="1">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>SourceSystem</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>'DBX' in France DBX partitions</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>EBP/OnPrem come from Synapse/on-prem partitions in same cube table.</t>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>EBP / OnPrem come from Synapse / on-prem partitions in the same cube table.</t>
         </is>
       </c>
     </row>
@@ -1829,484 +1827,462 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18.7109375" customWidth="1" min="1" max="1"/>
-    <col width="61.140625" customWidth="1" min="2" max="2"/>
-    <col width="42.7109375" customWidth="1" min="3" max="3"/>
-    <col width="9.140625" customWidth="1" min="4" max="4"/>
-    <col width="21.7109375" customWidth="1" min="5" max="5"/>
-    <col width="32" customWidth="1" min="6" max="6"/>
-    <col width="19.42578125" customWidth="1" min="7" max="7"/>
-    <col width="50.42578125" customWidth="1" min="8" max="8"/>
-    <col width="116.28515625" customWidth="1" min="9" max="9"/>
-    <col width="41.28515625" customWidth="1" min="10" max="10"/>
-    <col width="9.140625" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="8" max="8"/>
+    <col width="45" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Cube Name</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>KPI</t>
         </is>
       </c>
-      <c r="C1" s="5" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Problem </t>
         </is>
       </c>
-      <c r="D1" s="5" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Tester </t>
         </is>
       </c>
-      <c r="E1" s="5" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Responsible </t>
         </is>
       </c>
-      <c r="F1" s="5" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="G1" s="5" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Status </t>
         </is>
       </c>
-      <c r="H1" s="5" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Comment</t>
         </is>
       </c>
-      <c r="I1" s="5" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Link </t>
         </is>
       </c>
-      <c r="J1" s="5" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Validated &amp; Closed (Yes/No)</t>
         </is>
       </c>
-      <c r="K1" s="5" t="n"/>
-    </row>
-    <row r="2">
-      <c r="A2" s="5" t="inlineStr">
+    </row>
+    <row r="2" ht="55" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>France</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Inventory Units', 'Total Free Inventory', 'Inventory Units Actual'</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Total Free Inventory', 'Units Actual' KPI mismatches from the Synapse to Databricks</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Rajani</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>German</t>
         </is>
       </c>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>To-Do</t>
         </is>
       </c>
-      <c r="H2" s="5" t="n"/>
-      <c r="I2" s="5" t="inlineStr">
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>https://puma-all.atlassian.net/browse/UDPEBP-323</t>
         </is>
       </c>
-      <c r="J2" s="5" t="n"/>
-      <c r="K2" s="5" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="J2" s="2" t="n"/>
+    </row>
+    <row r="3" ht="55" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>France</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Inventory Units Actual', 'Inventory Units Old', 'Inventory Units  Next' ,'inventory Units Discontinued'</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Values are different from syn to dbx, but we when we summed up ,value equal to 'Inventory Units' total in their respective cubes.</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Rajani</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>German</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>To-Do</t>
         </is>
       </c>
-      <c r="H3" s="5" t="n"/>
-      <c r="I3" s="5" t="inlineStr">
+      <c r="H3" s="2" t="n"/>
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>[UDPEBP-324] UDP-France-'Inventory Units Actual', 'Inventory Units Old', 'Inventory Units Next' ,'inventory Units Discontinued' - Jira ALL</t>
         </is>
       </c>
-      <c r="J3" s="5" t="n"/>
-      <c r="K3" s="5" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="J3" s="2" t="n"/>
+    </row>
+    <row r="4" ht="55" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>France</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>inventory units LY,'inventory units  vs LY, inventory units  vs LY%</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Values are as expected </t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Rajani</t>
         </is>
       </c>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="5" t="n"/>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>To-Do</t>
         </is>
       </c>
-      <c r="H4" s="5" t="n"/>
-      <c r="I4" s="5" t="n"/>
-      <c r="J4" s="5" t="n"/>
-      <c r="K4" s="5" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="H4" s="2" t="n"/>
+      <c r="I4" s="2" t="n"/>
+      <c r="J4" s="2" t="n"/>
+    </row>
+    <row r="5" ht="55" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>France</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Inventory Gross</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Aggregated value is not showing up in dbx cube ,but it is there in synapse cube .</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>Rajani</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>Akshay</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>To-Do</t>
         </is>
       </c>
-      <c r="H5" s="5" t="n"/>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="H5" s="2" t="n"/>
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>[UDPEBP-325] UDP-Inventory-France-Inventory Gross-KPI Total not displaying in DBX cube. - Jira ALL</t>
         </is>
       </c>
-      <c r="J5" s="5" t="n"/>
-      <c r="K5" s="5" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="J5" s="2" t="n"/>
+    </row>
+    <row r="6" ht="55" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>France</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Inventory Units Delivery Date', 'Inventory Units Delivery Date LW', ,Inventory Units'</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">When we tested 'Inventory units' along with the 'Delivery Date' column , the values are different in DBX cube. </t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>Rajani</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>German</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>To-Do</t>
         </is>
       </c>
-      <c r="H6" s="5" t="n"/>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="H6" s="2" t="n"/>
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>[UDPEBP-326] UDP-France-'Delivery Date Units ' KPI Discrepencies between SYN and DBX Cubes.een - Jira ALL</t>
         </is>
       </c>
-      <c r="J6" s="5" t="n"/>
-      <c r="K6" s="5" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="J6" s="2" t="n"/>
+    </row>
+    <row r="7" ht="55" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>France</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>PRICECURRENCY field is missing for a significant portion of records</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>A significant portion of inventory records contain blank/null values in the PRICECURRENCY column, which may impact inventory valuation, reporting accuracy, and business validation activities.</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Rajani</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>German</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>In-Progress</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="n"/>
-      <c r="I7" s="5" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>In-Progress</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="n"/>
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>https://puma-all.atlassian.net/browse/UDPEBP-321</t>
         </is>
       </c>
-      <c r="J7" s="5" t="n"/>
-      <c r="K7" s="5" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="J7" s="2" t="n"/>
+    </row>
+    <row r="8" ht="55" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>France</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>Inventory Gross</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>While testing the inventory dbx cube, we found that for the inventory type='ALLOCATEDONHOLD','ALLOCATEDTODELIVERY', ‘ALLOCATEDTO STOCK’ are having no GROSS values even they count of UNITS in dbx cube.</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>Rajani</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>German</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>To-Do</t>
         </is>
       </c>
-      <c r="H8" s="5" t="n"/>
-      <c r="I8" s="5" t="inlineStr">
+      <c r="H8" s="2" t="n"/>
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>https://puma-all.atlassian.net/browse/UDPEBP-328</t>
         </is>
       </c>
-      <c r="J8" s="5" t="n"/>
-      <c r="K8" s="5" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="J8" s="2" t="n"/>
+    </row>
+    <row r="9" ht="55" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>France</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>Inventory Gross LY, Inventory Gross vs LY, Inventory Gross vs LY%</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>UDP-France-'Inventory Gross LY' KPI is not picking actual values for Year '2026' in both SYN and DBX</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>Rajani</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>German</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>In-Progress</t>
-        </is>
-      </c>
-      <c r="H9" s="5" t="n"/>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>In-Progress</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="n"/>
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>[UDPEBP-330] UDP-France-'Inventory Gross LY' KPI is not picking actual values for Year '2026' in both SYN and DBX - Jira ALL</t>
         </is>
       </c>
-      <c r="J9" s="5" t="n"/>
-      <c r="K9" s="5" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="n"/>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="5" t="n"/>
-      <c r="D10" s="5" t="n"/>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10" s="5" t="n"/>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="5" t="n"/>
-      <c r="I10" s="5" t="n"/>
-      <c r="J10" s="5" t="n"/>
-      <c r="K10" s="5" t="n"/>
-    </row>
-    <row r="11" ht="70" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="J9" s="2" t="n"/>
+    </row>
+    <row r="10" ht="55" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>France</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>Inventory Units (Unrestricted)</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>DBX Unrestricted higher than Synapse because special stock E is included in UNRESTRICTEDSTOCK (example 026404-01-150 FR04: DBX 6706 = 3506 blank + 3200 E). Synapse total matched blank special stock only.</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Natalia / Rajani / Torsten</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>DBX Unrestricted higher than Synapse because special stock E is included in UNRESTRICTEDSTOCK (blank special stock matches Synapse).</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Natalia / Rajani</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>German / Akshay</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>In-Progress</t>
-        </is>
-      </c>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>Details in KPIs List under DBX Backend Flow / Logic and Synapse vs DBX.</t>
-        </is>
-      </c>
-      <c r="I11" s="5" t="n"/>
-      <c r="J11" s="5" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>In-Progress</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Checked 026404-01-150 / FR04: Syn 3,506 vs DBX 6,706 (= 3,506 blank + 3,200 E @ 0006).</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="n"/>
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
+    <row r="11" ht="55" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>